<commit_message>
Fix Excel file handling test to write data to the correct worksheet
</commit_message>
<xml_diff>
--- a/fileupload/New Microsoft Excel Worksheet.xlsx
+++ b/fileupload/New Microsoft Excel Worksheet.xlsx
@@ -1,29 +1,41 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Sheet2" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="Sheet3" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="Sheet10" state="visible" r:id="rId7"/>
   </sheets>
-  <calcPr calcId="122211"/>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+  <si>
+    <t>Super King Lunch box 3 Containers Stainless Steel Offic...</t>
+  </si>
+  <si>
+    <t>₹207</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -53,7 +65,15 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -341,28 +361,47 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
 </file>
</xml_diff>